<commit_message>
fixed teacher dashboard logic
</commit_message>
<xml_diff>
--- a/uploads/teacher_subject_mapping.xlsx
+++ b/uploads/teacher_subject_mapping.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\float\data\input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\LATEST FINAL MINI PROJECT\uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A661C70-258F-45B3-AD2F-6E56F691DEA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{498AF2D3-0D1A-418E-9393-CD9EF17FE6B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{849BA79E-C918-47C8-A74D-3C07CE7264D9}"/>
   </bookViews>
@@ -27,8 +27,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -36,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="43">
   <si>
     <t>faculty</t>
   </si>
@@ -54,6 +52,117 @@
   </si>
   <si>
     <t>ESDE</t>
+  </si>
+  <si>
+    <t>TEJ</t>
+  </si>
+  <si>
+    <t>FOC</t>
+  </si>
+  <si>
+    <t>DBMS LAB</t>
+  </si>
+  <si>
+    <t>AAD</t>
+  </si>
+  <si>
+    <t>IT W/S</t>
+  </si>
+  <si>
+    <t>CP</t>
+  </si>
+  <si>
+    <t>COA</t>
+  </si>
+  <si>
+    <t>CG</t>
+  </si>
+  <si>
+    <t>KCJ</t>
+  </si>
+  <si>
+    <t>NJP</t>
+  </si>
+  <si>
+    <t>DC</t>
+  </si>
+  <si>
+    <t>MINI PROJECT</t>
+  </si>
+  <si>
+    <t>OS</t>
+  </si>
+  <si>
+    <t>OS LAB</t>
+  </si>
+  <si>
+    <t>THV</t>
+  </si>
+  <si>
+    <t>CD</t>
+  </si>
+  <si>
+    <t>N/W LAB</t>
+  </si>
+  <si>
+    <t>AIJ</t>
+  </si>
+  <si>
+    <t>CCV</t>
+  </si>
+  <si>
+    <t>CSA</t>
+  </si>
+  <si>
+    <t>CCW</t>
+  </si>
+  <si>
+    <t>ANG</t>
+  </si>
+  <si>
+    <t>IPR</t>
+  </si>
+  <si>
+    <t>SE</t>
+  </si>
+  <si>
+    <t>DIM</t>
+  </si>
+  <si>
+    <t>DM</t>
+  </si>
+  <si>
+    <t>PROJECT</t>
+  </si>
+  <si>
+    <t>DA</t>
+  </si>
+  <si>
+    <t>SWC</t>
+  </si>
+  <si>
+    <t>ACTIVITY HOUR</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> ACTIVITY HOUR</t>
+  </si>
+  <si>
+    <t>IOT</t>
+  </si>
+  <si>
+    <t>JRD</t>
+  </si>
+  <si>
+    <t>BCT</t>
+  </si>
+  <si>
+    <t>SPM</t>
+  </si>
+  <si>
+    <t>SPJ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DBMS  </t>
   </si>
 </sst>
 </file>
@@ -425,7 +534,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3EA82E80-2D75-4B50-B5E1-CCF49967776B}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B50"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
@@ -460,6 +569,374 @@
         <v>5</v>
       </c>
     </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>15</v>
+      </c>
+      <c r="B14" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>15</v>
+      </c>
+      <c r="B15" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>20</v>
+      </c>
+      <c r="B18" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>20</v>
+      </c>
+      <c r="B19" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>23</v>
+      </c>
+      <c r="B20" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>23</v>
+      </c>
+      <c r="B21" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>23</v>
+      </c>
+      <c r="B22" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>23</v>
+      </c>
+      <c r="B23" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>23</v>
+      </c>
+      <c r="B24" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>23</v>
+      </c>
+      <c r="B25" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>23</v>
+      </c>
+      <c r="B26" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>27</v>
+      </c>
+      <c r="B27" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>27</v>
+      </c>
+      <c r="B28" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>27</v>
+      </c>
+      <c r="B29" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>27</v>
+      </c>
+      <c r="B30" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>27</v>
+      </c>
+      <c r="B31" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>27</v>
+      </c>
+      <c r="B32" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>30</v>
+      </c>
+      <c r="B33" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>30</v>
+      </c>
+      <c r="B34" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>30</v>
+      </c>
+      <c r="B35" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>30</v>
+      </c>
+      <c r="B36" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>34</v>
+      </c>
+      <c r="B37" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>34</v>
+      </c>
+      <c r="B38" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>34</v>
+      </c>
+      <c r="B39" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>34</v>
+      </c>
+      <c r="B40" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>38</v>
+      </c>
+      <c r="B41" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>38</v>
+      </c>
+      <c r="B42" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>38</v>
+      </c>
+      <c r="B43" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>40</v>
+      </c>
+      <c r="B44" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>40</v>
+      </c>
+      <c r="B45" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>40</v>
+      </c>
+      <c r="B46" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>41</v>
+      </c>
+      <c r="B47" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>41</v>
+      </c>
+      <c r="B48" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>41</v>
+      </c>
+      <c r="B49" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>41</v>
+      </c>
+      <c r="B50" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
teacher dashboard partial fixed
</commit_message>
<xml_diff>
--- a/uploads/teacher_subject_mapping.xlsx
+++ b/uploads/teacher_subject_mapping.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\LATEST FINAL MINI PROJECT\uploads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{498AF2D3-0D1A-418E-9393-CD9EF17FE6B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C8775BA-1EF5-4987-A6AD-8D9D8B1EEC7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{849BA79E-C918-47C8-A74D-3C07CE7264D9}"/>
+    <workbookView xWindow="3312" yWindow="3312" windowWidth="17280" windowHeight="8880" xr2:uid="{849BA79E-C918-47C8-A74D-3C07CE7264D9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="47">
   <si>
     <t>faculty</t>
   </si>
@@ -42,18 +42,6 @@
     <t>subject</t>
   </si>
   <si>
-    <t>THERES</t>
-  </si>
-  <si>
-    <t>SAII</t>
-  </si>
-  <si>
-    <t>DDM</t>
-  </si>
-  <si>
-    <t>ESDE</t>
-  </si>
-  <si>
     <t>TEJ</t>
   </si>
   <si>
@@ -87,9 +75,6 @@
     <t>DC</t>
   </si>
   <si>
-    <t>MINI PROJECT</t>
-  </si>
-  <si>
     <t>OS</t>
   </si>
   <si>
@@ -111,9 +96,6 @@
     <t>CCV</t>
   </si>
   <si>
-    <t>CSA</t>
-  </si>
-  <si>
     <t>CCW</t>
   </si>
   <si>
@@ -163,6 +145,36 @@
   </si>
   <si>
     <t xml:space="preserve">DBMS  </t>
+  </si>
+  <si>
+    <t>class</t>
+  </si>
+  <si>
+    <t>S4_CSE_A</t>
+  </si>
+  <si>
+    <t>S6_CSE_B</t>
+  </si>
+  <si>
+    <t>S8_CSE</t>
+  </si>
+  <si>
+    <t>S2_CSE_A</t>
+  </si>
+  <si>
+    <t>S2_CSE_B</t>
+  </si>
+  <si>
+    <t>S4_CSE_B</t>
+  </si>
+  <si>
+    <t>S6_CSE_A</t>
+  </si>
+  <si>
+    <t>OS LAB/DBMS LAB</t>
+  </si>
+  <si>
+    <t>N/W LAB/MINI PROJECT</t>
   </si>
 </sst>
 </file>
@@ -534,407 +546,430 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3EA82E80-2D75-4B50-B5E1-CCF49967776B}">
-  <dimension ref="A1:B50"/>
+  <dimension ref="A1:C38"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="19.21875" customWidth="1"/>
+    <col min="3" max="3" width="12.21875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>2</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+        <v>45</v>
+      </c>
+      <c r="C3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>2</v>
       </c>
       <c r="B4" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" t="s">
         <v>6</v>
       </c>
-      <c r="B5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B6" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C6" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B7" t="s">
+        <v>45</v>
+      </c>
+      <c r="C7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C8" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" t="s">
+        <v>46</v>
+      </c>
+      <c r="C10" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
         <v>14</v>
       </c>
-      <c r="B9" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>14</v>
-      </c>
-      <c r="B10" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>14</v>
-      </c>
-      <c r="B11" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>14</v>
-      </c>
-      <c r="B12" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C12" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>15</v>
       </c>
       <c r="B13" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+      <c r="C13" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>15</v>
       </c>
       <c r="B14" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+        <v>16</v>
+      </c>
+      <c r="C14" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>15</v>
       </c>
       <c r="B15" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
         <v>18</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>15</v>
       </c>
       <c r="B16" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C16" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
+        <v>18</v>
+      </c>
+      <c r="B17" t="s">
         <v>20</v>
       </c>
-      <c r="B17" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C17" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B18" t="s">
+        <v>46</v>
+      </c>
+      <c r="C18" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>8</v>
+      </c>
+      <c r="C19" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>20</v>
-      </c>
-      <c r="B19" t="s">
+      <c r="B20" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
+      <c r="C20" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>21</v>
+      </c>
+      <c r="B21" t="s">
+        <v>30</v>
+      </c>
+      <c r="C21" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
         <v>23</v>
       </c>
-      <c r="B20" t="s">
+      <c r="C22" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>21</v>
+      </c>
+      <c r="B23" t="s">
+        <v>46</v>
+      </c>
+      <c r="C23" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>23</v>
-      </c>
-      <c r="B21" t="s">
+      <c r="B24" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>23</v>
-      </c>
-      <c r="B22" t="s">
+      <c r="C24" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>24</v>
+      </c>
+      <c r="B25" t="s">
+        <v>27</v>
+      </c>
+      <c r="C25" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>24</v>
+      </c>
+      <c r="B26" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>23</v>
-      </c>
-      <c r="B23" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
-        <v>23</v>
-      </c>
-      <c r="B24" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
-        <v>23</v>
-      </c>
-      <c r="B25" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
-        <v>23</v>
-      </c>
-      <c r="B26" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C26" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B27" t="s">
+        <v>46</v>
+      </c>
+      <c r="C27" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
-        <v>27</v>
-      </c>
       <c r="B28" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+      <c r="C28" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B29" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C29" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
+        <v>28</v>
+      </c>
+      <c r="B30" t="s">
+        <v>31</v>
+      </c>
+      <c r="C30" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>32</v>
+      </c>
+      <c r="B31" t="s">
+        <v>33</v>
+      </c>
+      <c r="C31" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>32</v>
+      </c>
+      <c r="B32" t="s">
+        <v>26</v>
+      </c>
+      <c r="C32" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>32</v>
+      </c>
+      <c r="B33" t="s">
         <v>27</v>
       </c>
-      <c r="B30" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
-        <v>27</v>
-      </c>
-      <c r="B31" t="s">
+      <c r="C33" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>34</v>
+      </c>
+      <c r="B34" t="s">
+        <v>16</v>
+      </c>
+      <c r="C34" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>34</v>
+      </c>
+      <c r="B35" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A32" t="s">
-        <v>27</v>
-      </c>
-      <c r="B32" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
-        <v>30</v>
-      </c>
-      <c r="B33" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A34" t="s">
-        <v>30</v>
-      </c>
-      <c r="B34" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A35" t="s">
-        <v>30</v>
-      </c>
-      <c r="B35" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C35" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B36" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+      <c r="C36" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B37" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+        <v>36</v>
+      </c>
+      <c r="C37" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B38" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A39" t="s">
-        <v>34</v>
-      </c>
-      <c r="B39" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A40" t="s">
-        <v>34</v>
-      </c>
-      <c r="B40" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A41" t="s">
-        <v>38</v>
-      </c>
-      <c r="B41" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A42" t="s">
-        <v>38</v>
-      </c>
-      <c r="B42" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A43" t="s">
-        <v>38</v>
-      </c>
-      <c r="B43" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A44" t="s">
-        <v>40</v>
-      </c>
-      <c r="B44" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A45" t="s">
-        <v>40</v>
-      </c>
-      <c r="B45" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A46" t="s">
-        <v>40</v>
-      </c>
-      <c r="B46" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A47" t="s">
-        <v>41</v>
-      </c>
-      <c r="B47" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A48" t="s">
-        <v>41</v>
-      </c>
-      <c r="B48" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A49" t="s">
-        <v>41</v>
-      </c>
-      <c r="B49" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A50" t="s">
-        <v>41</v>
-      </c>
-      <c r="B50" t="s">
-        <v>11</v>
+        <v>4</v>
+      </c>
+      <c r="C38" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
imporved export function and faculty list
</commit_message>
<xml_diff>
--- a/uploads/teacher_subject_mapping.xlsx
+++ b/uploads/teacher_subject_mapping.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C8775BA-1EF5-4987-A6AD-8D9D8B1EEC7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2AD86E4-A7D6-4AAF-A3ED-0B7FBEFA7AF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3312" yWindow="3312" windowWidth="17280" windowHeight="8880" xr2:uid="{849BA79E-C918-47C8-A74D-3C07CE7264D9}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{849BA79E-C918-47C8-A74D-3C07CE7264D9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="48">
   <si>
     <t>faculty</t>
   </si>
@@ -175,6 +175,9 @@
   </si>
   <si>
     <t>N/W LAB/MINI PROJECT</t>
+  </si>
+  <si>
+    <t>CSA</t>
   </si>
 </sst>
 </file>
@@ -546,7 +549,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3EA82E80-2D75-4B50-B5E1-CCF49967776B}">
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -724,7 +727,7 @@
         <v>18</v>
       </c>
       <c r="B16" t="s">
-        <v>19</v>
+        <v>47</v>
       </c>
       <c r="C16" t="s">
         <v>40</v>
@@ -790,10 +793,10 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C22" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
@@ -801,21 +804,21 @@
         <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="C23" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B24" t="s">
-        <v>25</v>
+        <v>46</v>
       </c>
       <c r="C24" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
@@ -823,10 +826,10 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C25" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
@@ -834,10 +837,10 @@
         <v>24</v>
       </c>
       <c r="B26" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C26" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
@@ -845,21 +848,21 @@
         <v>24</v>
       </c>
       <c r="B27" t="s">
-        <v>46</v>
+        <v>26</v>
       </c>
       <c r="C27" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B28" t="s">
-        <v>3</v>
+        <v>46</v>
       </c>
       <c r="C28" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
@@ -867,7 +870,7 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>29</v>
+        <v>3</v>
       </c>
       <c r="C29" t="s">
         <v>42</v>
@@ -878,18 +881,18 @@
         <v>28</v>
       </c>
       <c r="B30" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C30" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="B31" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C31" t="s">
         <v>40</v>
@@ -900,7 +903,7 @@
         <v>32</v>
       </c>
       <c r="B32" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="C32" t="s">
         <v>40</v>
@@ -911,18 +914,18 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C33" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B34" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="C34" t="s">
         <v>39</v>
@@ -933,7 +936,7 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C35" t="s">
         <v>39</v>
@@ -944,21 +947,21 @@
         <v>34</v>
       </c>
       <c r="B36" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="C36" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B37" t="s">
-        <v>36</v>
+        <v>7</v>
       </c>
       <c r="C37" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
@@ -966,9 +969,20 @@
         <v>35</v>
       </c>
       <c r="B38" t="s">
+        <v>36</v>
+      </c>
+      <c r="C38" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>35</v>
+      </c>
+      <c r="B39" t="s">
         <v>4</v>
       </c>
-      <c r="C38" t="s">
+      <c r="C39" t="s">
         <v>43</v>
       </c>
     </row>

</xml_diff>